<commit_message>
Fix skill-eval checkbox for plain-named NV Contests classes + remap DSA/DA modules
- Remove `want` filter (contest|test|neovarsity) when preferred_name is given so
  classes without those words in their name (e.g. "Advanced DSA 1", "Data Analytics
  and Visualisation - Fundamentals") can be found in NV Contests
- Fix applies to Playwright _find_target(), JS tryClick() scroll fallback, and
  the initial wait_for guard
- Remap Academy DSA modules to NV Contests: Advanced DSA 1-4, DSA 4.2,
  DSA for Competitive Programming, Data Structure Algorithms 1-4
- Remap Academy modules: Full-stack LLD and Development 4, Introduction to
  Problem Solving (Intermediate) 1, Data Engineering
- Remap DSML: Data Analytics and Visualisation - Fundamentals,
  Probability and Stats, Python Libraries to NV Contests

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Academy: Introduction to Problem Solving (Intermediate) 1 &amp; 2</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Academy: Data Structures and Algorithms (Beginner)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Academy: Data Structures and Algorithms (Beginner)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Academy: Data Structures and Algorithms (Beginner)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Academy: Data Structures and Algorithms (Beginner)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advanced DSA (Int/Adv)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advanced DSA (Int/Adv)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advanced DSA (Int/Adv)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advanced DSA (Int/Adv)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Academy: Full-stack LLD and Development 4</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Data Engineering New Nov25</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Academy: DSA 4.2</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Academy: DSA for Competitive Programming</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -1314,16 +1314,8 @@
       <c r="Z39" s="43" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>Data Engineering</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>Academy: Data Engineering (Old)</t>
-        </is>
-      </c>
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="9" t="n"/>
       <c r="C40" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/21</t>
@@ -1422,16 +1414,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>Data Engineering</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>Academy: Data Engineering (NA)</t>
-        </is>
-      </c>
+      <c r="A45" s="9" t="n"/>
+      <c r="B45" s="9" t="n"/>
       <c r="C45" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/532</t>
@@ -23887,7 +23871,11 @@
       <c r="C9" s="40" t="n">
         <v>71</v>
       </c>
-      <c r="D9" s="41" t="n"/>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/71</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="40" t="inlineStr">
@@ -23903,7 +23891,11 @@
       <c r="C10" s="40" t="n">
         <v>63</v>
       </c>
-      <c r="D10" s="41" t="n"/>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/63</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Remap Advance Software Engineering to NV Contests + add NV Contests fallback
- Excel: change 'Advance Software Engineering' library from
  'Academy: Advance Software Engineering (Beginner)' to 'NV Contests',
  matching the pattern used for DSA/LLD modules
- schedule_creator: extract library dropdown selection into
  _select_library_in_dropdown() helper
- schedule_creator: when _check_skill_eval_checkbox fails with the
  Excel-mapped library, automatically retry with 'NV Contests' before
  raising — handles any module not yet remapped in the Excel sheet

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -952,14 +952,10 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advance Software Engineering (Beginner)</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/410</t>
-        </is>
-      </c>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Remap AWS 1 and AWS 2 to NV Contests library
Both modules were mapped to bare 'AWS 1'/'AWS 2' library names which
only created 2 re-attempt slots in CCT instead of 4, causing the preview
to show 4 windows while Hire Test only received 2. NV Contests creates
4 attempts, matching the preview and all other NV contest modules.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -955,7 +955,11 @@
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C21" s="3" t="n"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/410</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1976,17 +1980,13 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>AWS 1</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C11" s="19" t="n">
         <v>592</v>
       </c>
-      <c r="D11" s="25" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/592</t>
-        </is>
-      </c>
+      <c r="D11" s="25" t="n"/>
       <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Live</t>
@@ -2024,17 +2024,13 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>AWS 2</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C12" s="19" t="n">
         <v>593</v>
       </c>
-      <c r="D12" s="25" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/593</t>
-        </is>
-      </c>
+      <c r="D12" s="25" t="n"/>
       <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Live</t>

</xml_diff>

<commit_message>
Add (AIML) suffix to GenAI/AI Agents modules; strip suffix before CCT matching
- 'Basics of GenAI and AI agents' and 'Advanced AI Agents' renamed to
  include '(AIML)' in AIML Libraries sheet so batch names are unambiguous
  when these modules appear in multiple programs.
- _check_skill_eval_checkbox now strips trailing parenthetical tags like
  '(AIML)' from preferred_name before matching against CCT class labels,
  so the CCT checkbox still matches correctly. Applies to all existing
  (AIML)-tagged modules (MLOPS, Maths for ML) too.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z46"/>
+  <dimension ref="A1:Z76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="40.88" customWidth="1" style="46" min="1" max="1"/>
@@ -597,6 +597,11 @@
           <t>Library Link</t>
         </is>
       </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>Num Attempts</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -633,77 +638,77 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Introduction to Programming (Beginner) 1</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Introduction to Programming (Beginner) 1 &amp; 2</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/278</t>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Introduction to Programming (Beginner) 1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Introduction to Programming (Beginner) 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/278</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
           <t>Introduction to Programming (Beginner) 2</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Introduction to Programming (Beginner) 1 &amp; 2</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/278</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Introduction to Problem Solving (Intermediate) 1</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/11</t>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Introduction to Problem Solving (Intermediate) 2</t>
+          <t>Introduction to Programming (Beginner) 2</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Academy: Introduction to Problem Solving (Intermediate) 1 &amp; 2</t>
+          <t>Academy: Introduction to Programming (Beginner) 1 &amp; 2</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/11</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/278</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t>Introduction to Problem Solving (Intermediate) 1</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -713,48 +718,48 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Data Structure Algorithms 2</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Introduction to Problem Solving (Intermediate) 2</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 3</t>
+          <t>Introduction to Problem Solving (Intermediate) 2</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>NV Contests</t>
+          <t>Academy: Introduction to Problem Solving (Intermediate) 1 &amp; 2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 4</t>
+          <t>Data Structure Algorithms 1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -771,7 +776,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Advanced DSA 1</t>
+          <t>Data Structure Algorithms 2</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -781,14 +786,14 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Advanced DSA 2</t>
+          <t>Data Structure Algorithms 3</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -798,14 +803,14 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Advanced DSA 3</t>
+          <t>Data Structure Algorithms 4</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -815,14 +820,14 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/281</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Advanced DSA 4</t>
+          <t>Advanced DSA 1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -839,603 +844,1131 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Databases &amp; SQL</t>
+          <t>Advanced DSA 2</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Academy: Databases and SQL (SEPT 2025)</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/713</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
-      <c r="L16" s="4" t="n"/>
-      <c r="M16" s="4" t="n"/>
-      <c r="N16" s="4" t="n"/>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="4" t="n"/>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="4" t="n"/>
-      <c r="T16" s="4" t="n"/>
-      <c r="U16" s="4" t="n"/>
-      <c r="V16" s="4" t="n"/>
-      <c r="W16" s="4" t="n"/>
-      <c r="X16" s="4" t="n"/>
-      <c r="Y16" s="4" t="n"/>
-      <c r="Z16" s="4" t="n"/>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Advance Programming Concepts</t>
+          <t>Advanced DSA 3</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Academy: Advance Programming Concepts (Beginner)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/343</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Advance Programming Concepts</t>
+          <t>Advanced DSA 4</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Academy: Python Advance Programming Concepts</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/417</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Low Level Design</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Low Level Design (Beginner)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/383</t>
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Databases &amp; SQL</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Low Level Design</t>
+          <t>Databases &amp; SQL</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Academy: Python Low Level Design (2024)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/423</t>
-        </is>
-      </c>
+          <t>Academy: Databases and SQL (SEPT 2025)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/713</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
+      <c r="N20" s="4" t="n"/>
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
+      <c r="T20" s="4" t="n"/>
+      <c r="U20" s="4" t="n"/>
+      <c r="V20" s="4" t="n"/>
+      <c r="W20" s="4" t="n"/>
+      <c r="X20" s="4" t="n"/>
+      <c r="Y20" s="4" t="n"/>
+      <c r="Z20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Advance Software Engineering</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Advance Programming Concepts</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/410</t>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Advance Software Engineering</t>
+          <t>Advance Programming Concepts</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Academy: Python Advance Software Engineering(2024)</t>
+          <t>Academy: Advance Programming Concepts (Beginner)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/467</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/343</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Backend Project</t>
+          <t>Advance Programming Concepts</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Academy: Backend Project (Beginner)</t>
+          <t>Academy: Python Advance Programming Concepts</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/320</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/417</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Backend Project</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Python Backend Project</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/398</t>
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Low Level Design</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Backend LLD and Development 1</t>
+          <t>Low Level Design</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Academy: Backend LLD 1,2,3</t>
+          <t>Academy: Low Level Design (Beginner)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/383</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Backend LLD and Development 2</t>
+          <t>Low Level Design</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Academy: Backend LLD 1,2,3</t>
+          <t>Academy: Python Low Level Design (2024)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/423</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Backend LLD and Development 3</t>
+          <t>Advance Software Engineering</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Academy: Backend LLD 1,2,3</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
-        </is>
+          <t>https://www.scaler.com/scm/classes/edit-library/410</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Backend Capstone Project</t>
+          <t>Advance Software Engineering</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Backend Capstone Project Latest (Dec2025)</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/757</t>
-        </is>
+          <t>Academy: Python Advance Software Engineering(2024)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/467</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Full-stack LLD and Development 1</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Full-stack LLD and Development 1</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/355</t>
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>Backend Project</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Full-stack LLD and Development 2</t>
+          <t>Backend Project</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Academy: Full-stack LLD and Development 2 (Beginners)</t>
+          <t>Academy: Backend Project (Beginner)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/356</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/320</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Full-stack LLD and Development 2</t>
+          <t>Backend Project</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Academy: Full-stack LLD and Development 2 (Int/Adv)</t>
+          <t>Academy: Python Backend Project</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/365</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/398</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Full-stack LLD and Development 3</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Academy: Full-stack LLD and Development 3</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/385</t>
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>Backend LLD and Development 1</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Full-stack LLD and Development 4</t>
+          <t>Backend LLD and Development 1</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
+          <t>Academy: Backend LLD 1,2,3</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>Backend LLD and Development 2</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/386</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>High Level Design</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Academy: HLD (New)</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/647</t>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Product Management for Software Engineers</t>
+          <t>Backend LLD and Development 2</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Academy: Product Management</t>
+          <t>Academy: Backend LLD 1,2,3</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/218</t>
-        </is>
+          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Data Engineering</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>Backend LLD and Development 3</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/751</t>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
+          <t>Backend LLD and Development 3</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Backend LLD 1,2,3</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/128</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>Backend Capstone Project</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Backend Capstone Project</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Backend Capstone Project Latest (Dec2025)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/757</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 1</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 1</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Full-stack LLD and Development 1</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/355</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 2</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 2</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Full-stack LLD and Development 2 (Beginners)</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/356</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 2</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Full-stack LLD and Development 2 (Int/Adv)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/365</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 3</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 3</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Full-stack LLD and Development 3</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/385</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack LLD and Development 4</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/386</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>High Level Design</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>High Level Design</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Academy: HLD (New)</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/647</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>Product Management for Software Engineers</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Product Management for Software Engineers</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Academy: Product Management</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/218</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Data Engineering</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/751</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
           <t>DSA 4.2</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/291</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>DSA for Competitive Programming</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/2</t>
         </is>
       </c>
-      <c r="D38" s="43" t="n"/>
-      <c r="E38" s="43" t="n"/>
-      <c r="F38" s="43" t="n"/>
-      <c r="G38" s="43" t="n"/>
-      <c r="H38" s="43" t="n"/>
-      <c r="I38" s="43" t="n"/>
-      <c r="J38" s="43" t="n"/>
-      <c r="K38" s="43" t="n"/>
-      <c r="L38" s="43" t="n"/>
-      <c r="M38" s="43" t="n"/>
-      <c r="N38" s="43" t="n"/>
-      <c r="O38" s="43" t="n"/>
-      <c r="P38" s="43" t="n"/>
-      <c r="Q38" s="43" t="n"/>
-      <c r="R38" s="43" t="n"/>
-      <c r="S38" s="43" t="n"/>
-      <c r="T38" s="43" t="n"/>
-      <c r="U38" s="43" t="n"/>
-      <c r="V38" s="43" t="n"/>
-      <c r="W38" s="43" t="n"/>
-      <c r="X38" s="43" t="n"/>
-      <c r="Y38" s="43" t="n"/>
-      <c r="Z38" s="43" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="D54" s="43" t="n"/>
+      <c r="E54" s="43" t="n"/>
+      <c r="F54" s="43" t="n"/>
+      <c r="G54" s="43" t="n"/>
+      <c r="H54" s="43" t="n"/>
+      <c r="I54" s="43" t="n"/>
+      <c r="J54" s="43" t="n"/>
+      <c r="K54" s="43" t="n"/>
+      <c r="L54" s="43" t="n"/>
+      <c r="M54" s="43" t="n"/>
+      <c r="N54" s="43" t="n"/>
+      <c r="O54" s="43" t="n"/>
+      <c r="P54" s="43" t="n"/>
+      <c r="Q54" s="43" t="n"/>
+      <c r="R54" s="43" t="n"/>
+      <c r="S54" s="43" t="n"/>
+      <c r="T54" s="43" t="n"/>
+      <c r="U54" s="43" t="n"/>
+      <c r="V54" s="43" t="n"/>
+      <c r="W54" s="43" t="n"/>
+      <c r="X54" s="43" t="n"/>
+      <c r="Y54" s="43" t="n"/>
+      <c r="Z54" s="43" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>Backend Capstone Project</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B55" s="9" t="inlineStr">
         <is>
           <t>Academy: Backend Capstone Project (Old-ongoing)</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/352</t>
         </is>
       </c>
-      <c r="D39" s="43" t="n"/>
-      <c r="E39" s="43" t="n"/>
-      <c r="F39" s="43" t="n"/>
-      <c r="G39" s="43" t="n"/>
-      <c r="H39" s="43" t="n"/>
-      <c r="I39" s="43" t="n"/>
-      <c r="J39" s="43" t="n"/>
-      <c r="K39" s="43" t="n"/>
-      <c r="L39" s="43" t="n"/>
-      <c r="M39" s="43" t="n"/>
-      <c r="N39" s="43" t="n"/>
-      <c r="O39" s="43" t="n"/>
-      <c r="P39" s="43" t="n"/>
-      <c r="Q39" s="43" t="n"/>
-      <c r="R39" s="43" t="n"/>
-      <c r="S39" s="43" t="n"/>
-      <c r="T39" s="43" t="n"/>
-      <c r="U39" s="43" t="n"/>
-      <c r="V39" s="43" t="n"/>
-      <c r="W39" s="43" t="n"/>
-      <c r="X39" s="43" t="n"/>
-      <c r="Y39" s="43" t="n"/>
-      <c r="Z39" s="43" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="9" t="n"/>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="D55" s="43" t="n"/>
+      <c r="E55" s="43" t="n"/>
+      <c r="F55" s="43" t="n"/>
+      <c r="G55" s="43" t="n"/>
+      <c r="H55" s="43" t="n"/>
+      <c r="I55" s="43" t="n"/>
+      <c r="J55" s="43" t="n"/>
+      <c r="K55" s="43" t="n"/>
+      <c r="L55" s="43" t="n"/>
+      <c r="M55" s="43" t="n"/>
+      <c r="N55" s="43" t="n"/>
+      <c r="O55" s="43" t="n"/>
+      <c r="P55" s="43" t="n"/>
+      <c r="Q55" s="43" t="n"/>
+      <c r="R55" s="43" t="n"/>
+      <c r="S55" s="43" t="n"/>
+      <c r="T55" s="43" t="n"/>
+      <c r="U55" s="43" t="n"/>
+      <c r="V55" s="43" t="n"/>
+      <c r="W55" s="43" t="n"/>
+      <c r="X55" s="43" t="n"/>
+      <c r="Y55" s="43" t="n"/>
+      <c r="Z55" s="43" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="n"/>
+      <c r="B56" s="9" t="n"/>
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/21</t>
         </is>
       </c>
-      <c r="D40" s="43" t="n"/>
-      <c r="E40" s="43" t="n"/>
-      <c r="F40" s="43" t="n"/>
-      <c r="G40" s="43" t="n"/>
-      <c r="H40" s="43" t="n"/>
-      <c r="I40" s="43" t="n"/>
-      <c r="J40" s="43" t="n"/>
-      <c r="K40" s="43" t="n"/>
-      <c r="L40" s="43" t="n"/>
-      <c r="M40" s="43" t="n"/>
-      <c r="N40" s="43" t="n"/>
-      <c r="O40" s="43" t="n"/>
-      <c r="P40" s="43" t="n"/>
-      <c r="Q40" s="43" t="n"/>
-      <c r="R40" s="43" t="n"/>
-      <c r="S40" s="43" t="n"/>
-      <c r="T40" s="43" t="n"/>
-      <c r="U40" s="43" t="n"/>
-      <c r="V40" s="43" t="n"/>
-      <c r="W40" s="43" t="n"/>
-      <c r="X40" s="43" t="n"/>
-      <c r="Y40" s="43" t="n"/>
-      <c r="Z40" s="43" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="D56" s="43" t="n"/>
+      <c r="E56" s="43" t="n"/>
+      <c r="F56" s="43" t="n"/>
+      <c r="G56" s="43" t="n"/>
+      <c r="H56" s="43" t="n"/>
+      <c r="I56" s="43" t="n"/>
+      <c r="J56" s="43" t="n"/>
+      <c r="K56" s="43" t="n"/>
+      <c r="L56" s="43" t="n"/>
+      <c r="M56" s="43" t="n"/>
+      <c r="N56" s="43" t="n"/>
+      <c r="O56" s="43" t="n"/>
+      <c r="P56" s="43" t="n"/>
+      <c r="Q56" s="43" t="n"/>
+      <c r="R56" s="43" t="n"/>
+      <c r="S56" s="43" t="n"/>
+      <c r="T56" s="43" t="n"/>
+      <c r="U56" s="43" t="n"/>
+      <c r="V56" s="43" t="n"/>
+      <c r="W56" s="43" t="n"/>
+      <c r="X56" s="43" t="n"/>
+      <c r="Y56" s="43" t="n"/>
+      <c r="Z56" s="43" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>High Level Design</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B57" s="9" t="inlineStr">
         <is>
           <t>Academy: HLD (Intermediate + Advanced + Beginner)</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/20</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
         <is>
           <t>Databases &amp; SQL</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B58" s="9" t="inlineStr">
         <is>
           <t>Academy: SQL (Oldv2)</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/408</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
         <is>
           <t>Databases &amp; SQL</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B59" s="9" t="inlineStr">
         <is>
           <t>Academy: SQL Inverted (NA)</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/409</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
         <is>
           <t>Backend Capstone Project</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Academy: Backend Capstone Project Inverted (NA) </t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/575</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="n"/>
-      <c r="B45" s="9" t="n"/>
-      <c r="C45" s="7" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="9" t="n"/>
+      <c r="B61" s="9" t="n"/>
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/532</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
         <is>
           <t>Backend Capstone Project</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>Academy: Backend Capstone Project (NA)</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/238</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t>Backend LLD and Development 4</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t>Advanced AI Agents</t>
+        </is>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t>Basics of GenAI and AI agents</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t>Common Core Fundamentals</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t>Common Core tools</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t>Common Core Foundations</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t>Common Core Maths</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t>Computer Systems and Fundamentals</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>LLD: Object Oriented Design and Analysis</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>LLD: Practical Software Engineering and Design</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>Full-Stack Capstone Project</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t>Full-stack Capstone Project</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t>Front-end Development</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t>Back-end development</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
@@ -1986,7 +2519,11 @@
       <c r="C11" s="19" t="n">
         <v>592</v>
       </c>
-      <c r="D11" s="25" t="n"/>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/592</t>
+        </is>
+      </c>
       <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Live</t>
@@ -2030,7 +2567,11 @@
       <c r="C12" s="19" t="n">
         <v>593</v>
       </c>
-      <c r="D12" s="25" t="n"/>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/593</t>
+        </is>
+      </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Live</t>
@@ -23601,7 +24142,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A1:Z44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="43" customWidth="1" style="46" min="1" max="1"/>
@@ -23666,46 +24207,24 @@
       <c r="Z1" s="37" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>SQL</t>
         </is>
       </c>
-      <c r="B2" s="38" t="inlineStr">
-        <is>
-          <t>SQL: New (DSML)</t>
-        </is>
-      </c>
-      <c r="C2" s="38" t="n">
-        <v>712</v>
-      </c>
-      <c r="D2" s="39" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/712</t>
-        </is>
-      </c>
-      <c r="E2" s="38" t="n"/>
-      <c r="F2" s="38" t="n"/>
-      <c r="G2" s="38" t="n"/>
-      <c r="H2" s="38" t="n"/>
-      <c r="I2" s="38" t="n"/>
-      <c r="J2" s="38" t="n"/>
-      <c r="K2" s="38" t="n"/>
-      <c r="L2" s="38" t="n"/>
-      <c r="M2" s="38" t="n"/>
-      <c r="N2" s="38" t="n"/>
-      <c r="O2" s="38" t="n"/>
-      <c r="P2" s="38" t="n"/>
-      <c r="Q2" s="38" t="n"/>
-      <c r="R2" s="38" t="n"/>
-      <c r="S2" s="38" t="n"/>
-      <c r="T2" s="38" t="n"/>
-      <c r="U2" s="38" t="n"/>
-      <c r="V2" s="38" t="n"/>
-      <c r="W2" s="38" t="n"/>
-      <c r="X2" s="38" t="n"/>
-      <c r="Y2" s="38" t="n"/>
-      <c r="Z2" s="38" t="n"/>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="38" t="inlineStr">
@@ -23715,15 +24234,15 @@
       </c>
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>Long-format SQL: New (DSML)</t>
+          <t>SQL: New (DSML)</t>
         </is>
       </c>
       <c r="C3" s="38" t="n">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="D3" s="39" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/717</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/712</t>
         </is>
       </c>
       <c r="E3" s="38" t="n"/>
@@ -23750,422 +24269,1475 @@
       <c r="Z3" s="38" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B4" s="38" t="inlineStr">
+        <is>
+          <t>Long-format SQL: New (DSML)</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="n">
+        <v>717</v>
+      </c>
+      <c r="D4" s="39" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/717</t>
+        </is>
+      </c>
+      <c r="E4" s="38" t="n"/>
+      <c r="F4" s="38" t="n"/>
+      <c r="G4" s="38" t="n"/>
+      <c r="H4" s="38" t="n"/>
+      <c r="I4" s="38" t="n"/>
+      <c r="J4" s="38" t="n"/>
+      <c r="K4" s="38" t="n"/>
+      <c r="L4" s="38" t="n"/>
+      <c r="M4" s="38" t="n"/>
+      <c r="N4" s="38" t="n"/>
+      <c r="O4" s="38" t="n"/>
+      <c r="P4" s="38" t="n"/>
+      <c r="Q4" s="38" t="n"/>
+      <c r="R4" s="38" t="n"/>
+      <c r="S4" s="38" t="n"/>
+      <c r="T4" s="38" t="n"/>
+      <c r="U4" s="38" t="n"/>
+      <c r="V4" s="38" t="n"/>
+      <c r="W4" s="38" t="n"/>
+      <c r="X4" s="38" t="n"/>
+      <c r="Y4" s="38" t="n"/>
+      <c r="Z4" s="38" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Tableau and Excel</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>Tableau and Excel</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>Tableau and Excel Long Version</t>
         </is>
       </c>
-      <c r="C4" s="40" t="n">
+      <c r="C6" s="40" t="n">
         <v>46</v>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/46</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>Tableau and Excel</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Tableau and Excel Short Version</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>638</v>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/638</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Beginner Python 1</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>Beginner Python 1</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Beginner Python 1 Inverted</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>172</v>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/172</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Beginner Python 2</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Beginner Python 2</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>Beginner Python 2 Inverted</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>561</v>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/561</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Data Analytics and Visualisation - Python Libraries</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Data Analytics and Visualisation - Python Libraries</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Data Analytics and Visualisation - Python Libraries</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>227</v>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/227</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>Data Analytics and Visualisation - Probability and Stats</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>71</v>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/71</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Data Analytics and Visualisation - Fundamentals</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>63</v>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/63</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>Product Analytics</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>Product Analytics</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Product Analytics</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>44</v>
+      </c>
+      <c r="D17" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/44</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Maths for ML</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>Maths for ML</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>Maths for ML</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>47</v>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/47</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>Intro to ML and NN</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/60</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>ML : Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>ML : Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="inlineStr">
+        <is>
+          <t>ML : Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="C22" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/52</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>ML : Adv Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>ML : Adv Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>ML : Adv Supervised Algorithms</t>
+        </is>
+      </c>
+      <c r="C24" s="40" t="n">
+        <v>414</v>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/414</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>ML : Unsupervised and RecSys</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>ML : Unsupervised and RecSys</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>ML : Unsupervised and RecSys</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="n">
+        <v>57</v>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/57</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>MLOps</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="40" t="inlineStr">
+        <is>
+          <t>MLOps</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t>MLOps</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="inlineStr">
+        <is>
+          <t>Neural Networks</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C29" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="D29" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/60</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="40" t="inlineStr">
+        <is>
+          <t>Computer Vision</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="D30" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/60</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="40" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="B32" s="40" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="C32" s="40" t="n">
+        <v>61</v>
+      </c>
+      <c r="D32" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/61</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>Advanced Python</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="40" t="inlineStr">
+        <is>
+          <t>Advanced Python</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="inlineStr">
+        <is>
+          <t>Advanced Python</t>
+        </is>
+      </c>
+      <c r="C34" s="40" t="n">
+        <v>56</v>
+      </c>
+      <c r="D34" s="42" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/56</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="inlineStr">
+        <is>
+          <t>DA Portfolio Project</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>DSML DA Portfolio Project</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="n">
+        <v>501</v>
+      </c>
+      <c r="D35" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/501</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="40" t="inlineStr">
+        <is>
+          <t>DS Portfolio Project</t>
+        </is>
+      </c>
+      <c r="B36" s="40" t="inlineStr">
+        <is>
+          <t>DSML DS Portfolio Project New</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>323</v>
+      </c>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/323</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="43" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B37" s="43" t="inlineStr">
+        <is>
+          <t>DSML Extra : SQL</t>
+        </is>
+      </c>
+      <c r="C37" s="43" t="n">
+        <v>97</v>
+      </c>
+      <c r="D37" s="44" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/97</t>
+        </is>
+      </c>
+      <c r="E37" s="43" t="n"/>
+      <c r="F37" s="43" t="n"/>
+      <c r="G37" s="43" t="n"/>
+      <c r="H37" s="43" t="n"/>
+      <c r="I37" s="43" t="n"/>
+      <c r="J37" s="43" t="n"/>
+      <c r="K37" s="43" t="n"/>
+      <c r="L37" s="43" t="n"/>
+      <c r="M37" s="43" t="n"/>
+      <c r="N37" s="43" t="n"/>
+      <c r="O37" s="43" t="n"/>
+      <c r="P37" s="43" t="n"/>
+      <c r="Q37" s="43" t="n"/>
+      <c r="R37" s="43" t="n"/>
+      <c r="S37" s="43" t="n"/>
+      <c r="T37" s="43" t="n"/>
+      <c r="U37" s="43" t="n"/>
+      <c r="V37" s="43" t="n"/>
+      <c r="W37" s="43" t="n"/>
+      <c r="X37" s="43" t="n"/>
+      <c r="Y37" s="43" t="n"/>
+      <c r="Z37" s="43" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="43" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B38" s="43" t="inlineStr">
+        <is>
+          <t>DSML Extra Misc</t>
+        </is>
+      </c>
+      <c r="C38" s="43" t="n">
+        <v>110</v>
+      </c>
+      <c r="D38" s="44" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/110</t>
+        </is>
+      </c>
+      <c r="E38" s="43" t="n"/>
+      <c r="F38" s="43" t="n"/>
+      <c r="G38" s="43" t="n"/>
+      <c r="H38" s="43" t="n"/>
+      <c r="I38" s="43" t="n"/>
+      <c r="J38" s="43" t="n"/>
+      <c r="K38" s="43" t="n"/>
+      <c r="L38" s="43" t="n"/>
+      <c r="M38" s="43" t="n"/>
+      <c r="N38" s="43" t="n"/>
+      <c r="O38" s="43" t="n"/>
+      <c r="P38" s="43" t="n"/>
+      <c r="Q38" s="43" t="n"/>
+      <c r="R38" s="43" t="n"/>
+      <c r="S38" s="43" t="n"/>
+      <c r="T38" s="43" t="n"/>
+      <c r="U38" s="43" t="n"/>
+      <c r="V38" s="43" t="n"/>
+      <c r="W38" s="43" t="n"/>
+      <c r="X38" s="43" t="n"/>
+      <c r="Y38" s="43" t="n"/>
+      <c r="Z38" s="43" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="43" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B39" s="43" t="inlineStr">
+        <is>
+          <t>SQL Library Long Version</t>
+        </is>
+      </c>
+      <c r="C39" s="43" t="n">
+        <v>165</v>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/165</t>
+        </is>
+      </c>
+      <c r="E39" s="43" t="n"/>
+      <c r="F39" s="43" t="n"/>
+      <c r="G39" s="43" t="n"/>
+      <c r="H39" s="43" t="n"/>
+      <c r="I39" s="43" t="n"/>
+      <c r="J39" s="43" t="n"/>
+      <c r="K39" s="43" t="n"/>
+      <c r="L39" s="43" t="n"/>
+      <c r="M39" s="43" t="n"/>
+      <c r="N39" s="43" t="n"/>
+      <c r="O39" s="43" t="n"/>
+      <c r="P39" s="43" t="n"/>
+      <c r="Q39" s="43" t="n"/>
+      <c r="R39" s="43" t="n"/>
+      <c r="S39" s="43" t="n"/>
+      <c r="T39" s="43" t="n"/>
+      <c r="U39" s="43" t="n"/>
+      <c r="V39" s="43" t="n"/>
+      <c r="W39" s="43" t="n"/>
+      <c r="X39" s="43" t="n"/>
+      <c r="Y39" s="43" t="n"/>
+      <c r="Z39" s="43" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="43" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B40" s="43" t="inlineStr">
+        <is>
+          <t>SQL Library Short Version</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="n">
+        <v>639</v>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/639</t>
+        </is>
+      </c>
+      <c r="E40" s="43" t="n"/>
+      <c r="F40" s="43" t="n"/>
+      <c r="G40" s="43" t="n"/>
+      <c r="H40" s="43" t="n"/>
+      <c r="I40" s="43" t="n"/>
+      <c r="J40" s="43" t="n"/>
+      <c r="K40" s="43" t="n"/>
+      <c r="L40" s="43" t="n"/>
+      <c r="M40" s="43" t="n"/>
+      <c r="N40" s="43" t="n"/>
+      <c r="O40" s="43" t="n"/>
+      <c r="P40" s="43" t="n"/>
+      <c r="Q40" s="43" t="n"/>
+      <c r="R40" s="43" t="n"/>
+      <c r="S40" s="43" t="n"/>
+      <c r="T40" s="43" t="n"/>
+      <c r="U40" s="43" t="n"/>
+      <c r="V40" s="43" t="n"/>
+      <c r="W40" s="43" t="n"/>
+      <c r="X40" s="43" t="n"/>
+      <c r="Y40" s="43" t="n"/>
+      <c r="Z40" s="43" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>Classical ML 1</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>DA ML 1</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>DA ML 2</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>Advanced SQL</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId25"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z24"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="42.25" customWidth="1" style="46" min="1" max="1"/>
+    <col width="77.5" customWidth="1" style="46" min="2" max="2"/>
+    <col width="48.88" customWidth="1" style="46" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Name </t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Library Name </t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Library id</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contest link </t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>Data Foundations</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Data Foundations</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>Data Foundations (Jan 2026)</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="n">
+        <v>768</v>
+      </c>
+      <c r="D3" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/768</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>ML Coding: Supervised Learning</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="40" t="inlineStr">
         <is>
-          <t>Tableau and Excel</t>
+          <t>ML Coding: Supervised Learning</t>
         </is>
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Tableau and Excel Short Version</t>
+          <t>ML Coding: Supervised Learning</t>
         </is>
       </c>
       <c r="C5" s="40" t="n">
-        <v>638</v>
+        <v>702</v>
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/638</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/702</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="inlineStr">
-        <is>
-          <t>Beginner Python 1</t>
-        </is>
-      </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>Beginner Python 1 Inverted</t>
-        </is>
-      </c>
-      <c r="C6" s="40" t="n">
-        <v>172</v>
-      </c>
-      <c r="D6" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/172</t>
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>ML Coding: Unsupervised Learning, Time series &amp; Recommender Systems</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="40" t="inlineStr">
         <is>
-          <t>Beginner Python 2</t>
+          <t>ML Coding: Unsupervised Learning, Time series &amp; Recommender Systems</t>
         </is>
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Beginner Python 2 Inverted</t>
+          <t>ML Coding: Unsupervised Learning, Time series &amp; Recommender Systems</t>
         </is>
       </c>
       <c r="C7" s="40" t="n">
-        <v>561</v>
+        <v>703</v>
       </c>
       <c r="D7" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/561</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/703</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr">
-        <is>
-          <t>Data Analytics and Visualisation - Python Libraries</t>
-        </is>
-      </c>
-      <c r="B8" s="40" t="inlineStr">
-        <is>
-          <t>Data Analytics and Visualisation - Python Libraries</t>
-        </is>
-      </c>
-      <c r="C8" s="40" t="n">
-        <v>227</v>
-      </c>
-      <c r="D8" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/227</t>
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>MLCoding: Neural Networks</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="40" t="inlineStr">
         <is>
-          <t>Data Analytics and Visualisation - Probability and Stats</t>
+          <t>MLCoding: Neural Networks</t>
         </is>
       </c>
       <c r="B9" s="40" t="inlineStr">
         <is>
+          <t>MLCoding: Neural Networks</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>704</v>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/704</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>MLCoding: Computer Vision and Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C9" s="40" t="n">
-        <v>71</v>
-      </c>
-      <c r="D9" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/71</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t>Data Analytics and Visualisation - Fundamentals</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>NV Contests</t>
-        </is>
-      </c>
-      <c r="C10" s="40" t="n">
-        <v>63</v>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/63</t>
+      <c r="C10" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="40" t="inlineStr">
         <is>
-          <t>Product Analytics</t>
+          <t>MLCoding: Computer Vision and Natural Language Processing</t>
         </is>
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>Product Analytics</t>
+          <t>MLCoding: Computer Vision and Natural Language Processing</t>
         </is>
       </c>
       <c r="C11" s="40" t="n">
-        <v>44</v>
+        <v>705</v>
       </c>
       <c r="D11" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/44</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/705</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="40" t="inlineStr">
         <is>
-          <t>Maths for ML</t>
+          <t>MLOPS (AIML)</t>
         </is>
       </c>
       <c r="B12" s="40" t="inlineStr">
         <is>
-          <t>Maths for ML</t>
+          <t>MLOPS (AIML)</t>
         </is>
       </c>
       <c r="C12" s="40" t="n">
-        <v>47</v>
+        <v>706</v>
       </c>
       <c r="D12" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/47</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/706</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="40" t="inlineStr">
         <is>
-          <t>Intro to ML and NN</t>
+          <t>ML System Design</t>
         </is>
       </c>
       <c r="B13" s="40" t="inlineStr">
         <is>
-          <t>Intro to ML and NN</t>
+          <t>ML System Design</t>
         </is>
       </c>
       <c r="C13" s="40" t="n">
-        <v>36</v>
+        <v>707</v>
       </c>
       <c r="D13" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/36</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/707</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="inlineStr">
-        <is>
-          <t>ML : Supervised Algorithms</t>
-        </is>
-      </c>
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t>ML : Supervised Algorithms</t>
-        </is>
-      </c>
-      <c r="C14" s="40" t="n">
-        <v>52</v>
-      </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/52</t>
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Basics of GenAI and AI agents (AIML)</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="40" t="inlineStr">
         <is>
-          <t>ML : Adv Supervised Algorithms</t>
+          <t>Basics of GenAI and AI agents (AIML)</t>
         </is>
       </c>
       <c r="B15" s="40" t="inlineStr">
         <is>
-          <t>ML : Adv Supervised Algorithms</t>
+          <t>Basics of GenAI and AI agents</t>
         </is>
       </c>
       <c r="C15" s="40" t="n">
-        <v>414</v>
+        <v>708</v>
       </c>
       <c r="D15" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/414</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/708</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="40" t="inlineStr">
-        <is>
-          <t>ML : Unsupervised and RecSys</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>ML : Unsupervised and RecSys</t>
-        </is>
-      </c>
-      <c r="C16" s="40" t="n">
-        <v>57</v>
-      </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/57</t>
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>Advanced AI Agents (AIML)</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="40" t="inlineStr">
         <is>
-          <t>MLOps</t>
+          <t>Advanced AI Agents (AIML)</t>
         </is>
       </c>
       <c r="B17" s="40" t="inlineStr">
         <is>
-          <t>MLOps</t>
+          <t>Advanced AI Agents</t>
         </is>
       </c>
       <c r="C17" s="40" t="n">
-        <v>50</v>
+        <v>709</v>
       </c>
       <c r="D17" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/50</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/709</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="40" t="inlineStr">
         <is>
-          <t>Neural Networks</t>
+          <t>LLMOPS (Recorded)</t>
         </is>
       </c>
       <c r="B18" s="40" t="inlineStr">
         <is>
-          <t>Neural Networks</t>
+          <t>LLMOPS (Recorded)</t>
         </is>
       </c>
       <c r="C18" s="40" t="n">
-        <v>58</v>
+        <v>710</v>
       </c>
       <c r="D18" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/58</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/710</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="40" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Reinforcement learning</t>
         </is>
       </c>
       <c r="B19" s="40" t="inlineStr">
         <is>
-          <t>Computer Vision</t>
+          <t>Reinforcement learning</t>
         </is>
       </c>
       <c r="C19" s="40" t="n">
-        <v>60</v>
+        <v>711</v>
       </c>
       <c r="D19" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/60</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/711</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="40" t="inlineStr">
         <is>
-          <t>Natural Language Processing</t>
+          <t>DSA for Professionals 1,2,3,4</t>
         </is>
       </c>
       <c r="B20" s="40" t="inlineStr">
         <is>
-          <t>Natural Language Processing</t>
+          <t>DSA for Professionals 1,2,3,4</t>
         </is>
       </c>
       <c r="C20" s="40" t="n">
-        <v>61</v>
-      </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/61</t>
+        <v>630</v>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/630</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="40" t="inlineStr">
         <is>
-          <t>Advanced Python</t>
+          <t>Agentic AI Systems</t>
         </is>
       </c>
       <c r="B21" s="40" t="inlineStr">
         <is>
-          <t>Advanced Python</t>
+          <t>AIML : Agentic AI Systems (Feb 2026)</t>
         </is>
       </c>
       <c r="C21" s="40" t="n">
-        <v>56</v>
+        <v>786</v>
       </c>
       <c r="D21" s="42" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/56</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/786</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
-        <is>
-          <t>DA Portfolio Project</t>
-        </is>
-      </c>
-      <c r="B22" s="40" t="inlineStr">
-        <is>
-          <t>DSML DA Portfolio Project</t>
-        </is>
-      </c>
-      <c r="C22" s="40" t="n">
-        <v>501</v>
-      </c>
-      <c r="D22" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/501</t>
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Maths for ML (AIML)</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="40" t="inlineStr">
         <is>
-          <t>DS Portfolio Project</t>
+          <t>Maths for ML (AIML)</t>
         </is>
       </c>
       <c r="B23" s="40" t="inlineStr">
         <is>
-          <t>DSML DS Portfolio Project New</t>
+          <t>AIML Maths for ML</t>
         </is>
       </c>
       <c r="C23" s="40" t="n">
-        <v>323</v>
-      </c>
-      <c r="D23" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/323</t>
+        <v>602</v>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/602</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="43" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>Data Foundations</t>
         </is>
       </c>
       <c r="B24" s="43" t="inlineStr">
         <is>
-          <t>DSML Extra : SQL</t>
+          <t>Data Foundations (NA)</t>
         </is>
       </c>
       <c r="C24" s="43" t="n">
-        <v>97</v>
+        <v>701</v>
       </c>
       <c r="D24" s="44" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/97</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/701</t>
         </is>
       </c>
       <c r="E24" s="43" t="n"/>
@@ -24190,538 +25762,6 @@
       <c r="X24" s="43" t="n"/>
       <c r="Y24" s="43" t="n"/>
       <c r="Z24" s="43" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="43" t="inlineStr">
-        <is>
-          <t>Misc</t>
-        </is>
-      </c>
-      <c r="B25" s="43" t="inlineStr">
-        <is>
-          <t>DSML Extra Misc</t>
-        </is>
-      </c>
-      <c r="C25" s="43" t="n">
-        <v>110</v>
-      </c>
-      <c r="D25" s="44" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/110</t>
-        </is>
-      </c>
-      <c r="E25" s="43" t="n"/>
-      <c r="F25" s="43" t="n"/>
-      <c r="G25" s="43" t="n"/>
-      <c r="H25" s="43" t="n"/>
-      <c r="I25" s="43" t="n"/>
-      <c r="J25" s="43" t="n"/>
-      <c r="K25" s="43" t="n"/>
-      <c r="L25" s="43" t="n"/>
-      <c r="M25" s="43" t="n"/>
-      <c r="N25" s="43" t="n"/>
-      <c r="O25" s="43" t="n"/>
-      <c r="P25" s="43" t="n"/>
-      <c r="Q25" s="43" t="n"/>
-      <c r="R25" s="43" t="n"/>
-      <c r="S25" s="43" t="n"/>
-      <c r="T25" s="43" t="n"/>
-      <c r="U25" s="43" t="n"/>
-      <c r="V25" s="43" t="n"/>
-      <c r="W25" s="43" t="n"/>
-      <c r="X25" s="43" t="n"/>
-      <c r="Y25" s="43" t="n"/>
-      <c r="Z25" s="43" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="43" t="inlineStr">
-        <is>
-          <t>SQL</t>
-        </is>
-      </c>
-      <c r="B26" s="43" t="inlineStr">
-        <is>
-          <t>SQL Library Long Version</t>
-        </is>
-      </c>
-      <c r="C26" s="43" t="n">
-        <v>165</v>
-      </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/165</t>
-        </is>
-      </c>
-      <c r="E26" s="43" t="n"/>
-      <c r="F26" s="43" t="n"/>
-      <c r="G26" s="43" t="n"/>
-      <c r="H26" s="43" t="n"/>
-      <c r="I26" s="43" t="n"/>
-      <c r="J26" s="43" t="n"/>
-      <c r="K26" s="43" t="n"/>
-      <c r="L26" s="43" t="n"/>
-      <c r="M26" s="43" t="n"/>
-      <c r="N26" s="43" t="n"/>
-      <c r="O26" s="43" t="n"/>
-      <c r="P26" s="43" t="n"/>
-      <c r="Q26" s="43" t="n"/>
-      <c r="R26" s="43" t="n"/>
-      <c r="S26" s="43" t="n"/>
-      <c r="T26" s="43" t="n"/>
-      <c r="U26" s="43" t="n"/>
-      <c r="V26" s="43" t="n"/>
-      <c r="W26" s="43" t="n"/>
-      <c r="X26" s="43" t="n"/>
-      <c r="Y26" s="43" t="n"/>
-      <c r="Z26" s="43" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="43" t="inlineStr">
-        <is>
-          <t>SQL</t>
-        </is>
-      </c>
-      <c r="B27" s="43" t="inlineStr">
-        <is>
-          <t>SQL Library Short Version</t>
-        </is>
-      </c>
-      <c r="C27" s="43" t="n">
-        <v>639</v>
-      </c>
-      <c r="D27" s="44" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/639</t>
-        </is>
-      </c>
-      <c r="E27" s="43" t="n"/>
-      <c r="F27" s="43" t="n"/>
-      <c r="G27" s="43" t="n"/>
-      <c r="H27" s="43" t="n"/>
-      <c r="I27" s="43" t="n"/>
-      <c r="J27" s="43" t="n"/>
-      <c r="K27" s="43" t="n"/>
-      <c r="L27" s="43" t="n"/>
-      <c r="M27" s="43" t="n"/>
-      <c r="N27" s="43" t="n"/>
-      <c r="O27" s="43" t="n"/>
-      <c r="P27" s="43" t="n"/>
-      <c r="Q27" s="43" t="n"/>
-      <c r="R27" s="43" t="n"/>
-      <c r="S27" s="43" t="n"/>
-      <c r="T27" s="43" t="n"/>
-      <c r="U27" s="43" t="n"/>
-      <c r="V27" s="43" t="n"/>
-      <c r="W27" s="43" t="n"/>
-      <c r="X27" s="43" t="n"/>
-      <c r="Y27" s="43" t="n"/>
-      <c r="Z27" s="43" t="n"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Z16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="42.25" customWidth="1" style="46" min="1" max="1"/>
-    <col width="77.5" customWidth="1" style="46" min="2" max="2"/>
-    <col width="48.88" customWidth="1" style="46" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Name </t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Library Name </t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Library id</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contest link </t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Months</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>Data Foundations</t>
-        </is>
-      </c>
-      <c r="B2" s="40" t="inlineStr">
-        <is>
-          <t>Data Foundations (Jan 2026)</t>
-        </is>
-      </c>
-      <c r="C2" s="40" t="n">
-        <v>768</v>
-      </c>
-      <c r="D2" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/768</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="40" t="inlineStr">
-        <is>
-          <t>ML Coding: Supervised Learning</t>
-        </is>
-      </c>
-      <c r="B3" s="40" t="inlineStr">
-        <is>
-          <t>ML Coding: Supervised Learning</t>
-        </is>
-      </c>
-      <c r="C3" s="40" t="n">
-        <v>702</v>
-      </c>
-      <c r="D3" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/702</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="40" t="inlineStr">
-        <is>
-          <t>ML Coding: Unsupervised Learning, Time series &amp; Recommender Systems</t>
-        </is>
-      </c>
-      <c r="B4" s="40" t="inlineStr">
-        <is>
-          <t>ML Coding: Unsupervised Learning, Time series &amp; Recommender Systems</t>
-        </is>
-      </c>
-      <c r="C4" s="40" t="n">
-        <v>703</v>
-      </c>
-      <c r="D4" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/703</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="40" t="inlineStr">
-        <is>
-          <t>MLCoding: Neural Networks</t>
-        </is>
-      </c>
-      <c r="B5" s="40" t="inlineStr">
-        <is>
-          <t>MLCoding: Neural Networks</t>
-        </is>
-      </c>
-      <c r="C5" s="40" t="n">
-        <v>704</v>
-      </c>
-      <c r="D5" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/704</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="40" t="inlineStr">
-        <is>
-          <t>MLCoding: Computer Vision and Natural Language Processing</t>
-        </is>
-      </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>MLCoding: Computer Vision and Natural Language Processing</t>
-        </is>
-      </c>
-      <c r="C6" s="40" t="n">
-        <v>705</v>
-      </c>
-      <c r="D6" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/705</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="40" t="inlineStr">
-        <is>
-          <t>MLOPS (AIML)</t>
-        </is>
-      </c>
-      <c r="B7" s="40" t="inlineStr">
-        <is>
-          <t>MLOPS (AIML)</t>
-        </is>
-      </c>
-      <c r="C7" s="40" t="n">
-        <v>706</v>
-      </c>
-      <c r="D7" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/706</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="40" t="inlineStr">
-        <is>
-          <t>ML System Design</t>
-        </is>
-      </c>
-      <c r="B8" s="40" t="inlineStr">
-        <is>
-          <t>ML System Design</t>
-        </is>
-      </c>
-      <c r="C8" s="40" t="n">
-        <v>707</v>
-      </c>
-      <c r="D8" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/707</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="40" t="inlineStr">
-        <is>
-          <t>Basics of GenAI and AI agents</t>
-        </is>
-      </c>
-      <c r="B9" s="40" t="inlineStr">
-        <is>
-          <t>Basics of GenAI and AI agents</t>
-        </is>
-      </c>
-      <c r="C9" s="40" t="n">
-        <v>708</v>
-      </c>
-      <c r="D9" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/708</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t>Advanced AI Agents</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Advanced AI Agents</t>
-        </is>
-      </c>
-      <c r="C10" s="40" t="n">
-        <v>709</v>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/709</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t>LLMOPS (Recorded)</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>LLMOPS (Recorded)</t>
-        </is>
-      </c>
-      <c r="C11" s="40" t="n">
-        <v>710</v>
-      </c>
-      <c r="D11" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/710</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="40" t="inlineStr">
-        <is>
-          <t>Reinforcement learning</t>
-        </is>
-      </c>
-      <c r="B12" s="40" t="inlineStr">
-        <is>
-          <t>Reinforcement learning</t>
-        </is>
-      </c>
-      <c r="C12" s="40" t="n">
-        <v>711</v>
-      </c>
-      <c r="D12" s="41" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/711</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>DSA for Professionals 1,2,3,4</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>DSA for Professionals 1,2,3,4</t>
-        </is>
-      </c>
-      <c r="C13" s="40" t="n">
-        <v>630</v>
-      </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/630</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="40" t="inlineStr">
-        <is>
-          <t>Agentic AI Systems</t>
-        </is>
-      </c>
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t>AIML : Agentic AI Systems (Feb 2026)</t>
-        </is>
-      </c>
-      <c r="C14" s="40" t="n">
-        <v>786</v>
-      </c>
-      <c r="D14" s="42" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/786</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t>Maths for ML (AIML)</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>AIML Maths for ML</t>
-        </is>
-      </c>
-      <c r="C15" s="40" t="n">
-        <v>602</v>
-      </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/602</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>Data Foundations</t>
-        </is>
-      </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>Data Foundations (NA)</t>
-        </is>
-      </c>
-      <c r="C16" s="43" t="n">
-        <v>701</v>
-      </c>
-      <c r="D16" s="44" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/701</t>
-        </is>
-      </c>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="43" t="n"/>
-      <c r="G16" s="43" t="n"/>
-      <c r="H16" s="43" t="n"/>
-      <c r="I16" s="43" t="n"/>
-      <c r="J16" s="43" t="n"/>
-      <c r="K16" s="43" t="n"/>
-      <c r="L16" s="43" t="n"/>
-      <c r="M16" s="43" t="n"/>
-      <c r="N16" s="43" t="n"/>
-      <c r="O16" s="43" t="n"/>
-      <c r="P16" s="43" t="n"/>
-      <c r="Q16" s="43" t="n"/>
-      <c r="R16" s="43" t="n"/>
-      <c r="S16" s="43" t="n"/>
-      <c r="T16" s="43" t="n"/>
-      <c r="U16" s="43" t="n"/>
-      <c r="V16" s="43" t="n"/>
-      <c r="W16" s="43" t="n"/>
-      <c r="X16" s="43" t="n"/>
-      <c r="Y16" s="43" t="n"/>
-      <c r="Z16" s="43" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Set NV Contests as default library for DevOps Linux 2 module
Prepends an NV Contests (library 338) row for "Linux Shell Scripting
and Computer Systems 2" in the DevOps sheet, ahead of the existing
DevOps: Linux 2 (Dec25)/(New) and Old candidates. Library 338 is the
shared multi-purpose NV Contests library already used across dozens
of academy/dsml/aiml contests per the metadata history.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2031,7 +2031,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1007"/>
+  <dimension ref="A1:Z1008"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="41.63" customWidth="1" style="46" min="1" max="1"/>
@@ -2096,50 +2096,29 @@
       <c r="Z1" s="38" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Beginner Python </t>
-        </is>
-      </c>
-      <c r="B2" s="24" t="inlineStr">
-        <is>
-          <t>Devops: Beginner Python (New)</t>
-        </is>
-      </c>
-      <c r="C2" s="19" t="n">
-        <v>653</v>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/653</t>
-        </is>
-      </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Linux Shell Scripting and Computer Systems 2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>338</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
       </c>
-      <c r="F2" s="24" t="n"/>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="38" t="n"/>
-      <c r="I2" s="38" t="n"/>
-      <c r="J2" s="38" t="n"/>
-      <c r="K2" s="38" t="n"/>
-      <c r="L2" s="38" t="n"/>
-      <c r="M2" s="38" t="n"/>
-      <c r="N2" s="38" t="n"/>
-      <c r="O2" s="38" t="n"/>
-      <c r="P2" s="38" t="n"/>
-      <c r="Q2" s="38" t="n"/>
-      <c r="R2" s="38" t="n"/>
-      <c r="S2" s="38" t="n"/>
-      <c r="T2" s="38" t="n"/>
-      <c r="U2" s="38" t="n"/>
-      <c r="V2" s="38" t="n"/>
-      <c r="W2" s="38" t="n"/>
-      <c r="X2" s="38" t="n"/>
-      <c r="Y2" s="38" t="n"/>
-      <c r="Z2" s="38" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
@@ -2149,18 +2128,18 @@
       </c>
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t>Devops: Beginner Python with Breaks (New)</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="n">
-        <v>667</v>
+          <t>Devops: Beginner Python (New)</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>653</v>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/667</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
+          <t>https://www.scaler.com/scm/classes/edit-library/653</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -2190,20 +2169,20 @@
     <row r="4">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t xml:space="preserve">Beginner Python </t>
         </is>
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>DevOps: DSA 1 (New)</t>
+          <t>Devops: Beginner Python with Breaks (New)</t>
         </is>
       </c>
       <c r="C4" s="17" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/666</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/667</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
@@ -2241,18 +2220,18 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>DevOps: DSA 1 with Breaks (New)</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>652</v>
+          <t>DevOps: DSA 1 (New)</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>666</v>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/652</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
+          <t>https://www.scaler.com/scm/classes/edit-library/666</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -2282,20 +2261,20 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 1</t>
-        </is>
-      </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>DevOps: Linux 1 (Dec25)</t>
+          <t>Data Structure Algorithms 1</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>DevOps: DSA 1 with Breaks (New)</t>
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>752</v>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/752</t>
+        <v>652</v>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/652</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
@@ -2305,43 +2284,43 @@
       </c>
       <c r="F6" s="24" t="n"/>
       <c r="G6" s="16" t="n"/>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="22" t="n"/>
-      <c r="J6" s="22" t="n"/>
-      <c r="K6" s="22" t="n"/>
-      <c r="L6" s="22" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="22" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="22" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="22" t="n"/>
-      <c r="T6" s="22" t="n"/>
-      <c r="U6" s="22" t="n"/>
-      <c r="V6" s="22" t="n"/>
-      <c r="W6" s="22" t="n"/>
-      <c r="X6" s="22" t="n"/>
-      <c r="Y6" s="22" t="n"/>
-      <c r="Z6" s="22" t="n"/>
+      <c r="H6" s="38" t="n"/>
+      <c r="I6" s="38" t="n"/>
+      <c r="J6" s="38" t="n"/>
+      <c r="K6" s="38" t="n"/>
+      <c r="L6" s="38" t="n"/>
+      <c r="M6" s="38" t="n"/>
+      <c r="N6" s="38" t="n"/>
+      <c r="O6" s="38" t="n"/>
+      <c r="P6" s="38" t="n"/>
+      <c r="Q6" s="38" t="n"/>
+      <c r="R6" s="38" t="n"/>
+      <c r="S6" s="38" t="n"/>
+      <c r="T6" s="38" t="n"/>
+      <c r="U6" s="38" t="n"/>
+      <c r="V6" s="38" t="n"/>
+      <c r="W6" s="38" t="n"/>
+      <c r="X6" s="38" t="n"/>
+      <c r="Y6" s="38" t="n"/>
+      <c r="Z6" s="38" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 2</t>
+          <t>Linux Shell Scripting and Computer Systems 1</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>DevOps: Linux 2 (Dec25)</t>
+          <t>DevOps: Linux 1 (Dec25)</t>
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>753</v>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/753</t>
+        <v>752</v>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/752</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
@@ -2351,43 +2330,43 @@
       </c>
       <c r="F7" s="24" t="n"/>
       <c r="G7" s="16" t="n"/>
-      <c r="H7" s="38" t="n"/>
-      <c r="I7" s="38" t="n"/>
-      <c r="J7" s="38" t="n"/>
-      <c r="K7" s="38" t="n"/>
-      <c r="L7" s="38" t="n"/>
-      <c r="M7" s="38" t="n"/>
-      <c r="N7" s="38" t="n"/>
-      <c r="O7" s="38" t="n"/>
-      <c r="P7" s="38" t="n"/>
-      <c r="Q7" s="38" t="n"/>
-      <c r="R7" s="38" t="n"/>
-      <c r="S7" s="38" t="n"/>
-      <c r="T7" s="38" t="n"/>
-      <c r="U7" s="38" t="n"/>
-      <c r="V7" s="38" t="n"/>
-      <c r="W7" s="38" t="n"/>
-      <c r="X7" s="38" t="n"/>
-      <c r="Y7" s="38" t="n"/>
-      <c r="Z7" s="38" t="n"/>
+      <c r="H7" s="22" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="22" t="n"/>
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="22" t="n"/>
+      <c r="O7" s="22" t="n"/>
+      <c r="P7" s="22" t="n"/>
+      <c r="Q7" s="22" t="n"/>
+      <c r="R7" s="22" t="n"/>
+      <c r="S7" s="22" t="n"/>
+      <c r="T7" s="22" t="n"/>
+      <c r="U7" s="22" t="n"/>
+      <c r="V7" s="22" t="n"/>
+      <c r="W7" s="22" t="n"/>
+      <c r="X7" s="22" t="n"/>
+      <c r="Y7" s="22" t="n"/>
+      <c r="Z7" s="22" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>DevOps Tools 1</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>DevOps: DevOps Tools 1 (New)</t>
+          <t>Linux Shell Scripting and Computer Systems 2</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>DevOps: Linux 2 (Dec25)</t>
         </is>
       </c>
       <c r="C8" s="19" t="n">
-        <v>674</v>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/674</t>
+        <v>753</v>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/753</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
@@ -2420,20 +2399,20 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>DevOps Tools 2</t>
+          <t>DevOps Tools 1</t>
         </is>
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>DevOps: DevOps Tools 2 (New)</t>
+          <t>DevOps: DevOps Tools 1 (New)</t>
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/676</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/674</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
@@ -2466,25 +2445,29 @@
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>Career Readiness</t>
+          <t>DevOps Tools 2</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>DevOps: Career Readiness Contest</t>
+          <t>DevOps: DevOps Tools 2 (New)</t>
         </is>
       </c>
       <c r="C10" s="19" t="n">
-        <v>754</v>
+        <v>676</v>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/754</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="n"/>
+          <t>https://www.scaler.com/scm/classes/edit-library/676</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="F10" s="24" t="n"/>
-      <c r="G10" s="17" t="n"/>
+      <c r="G10" s="16" t="n"/>
       <c r="H10" s="38" t="n"/>
       <c r="I10" s="38" t="n"/>
       <c r="J10" s="38" t="n"/>
@@ -2508,31 +2491,25 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>AWS 1</t>
+          <t>Career Readiness</t>
         </is>
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>NV Contests</t>
+          <t>DevOps: Career Readiness Contest</t>
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>592</v>
-      </c>
-      <c r="D11" s="25" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/592</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
+        <v>754</v>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/754</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="n"/>
       <c r="F11" s="24" t="n"/>
-      <c r="G11" s="19" t="n">
-        <v>2</v>
-      </c>
+      <c r="G11" s="17" t="n"/>
       <c r="H11" s="38" t="n"/>
       <c r="I11" s="38" t="n"/>
       <c r="J11" s="38" t="n"/>
@@ -2556,7 +2533,7 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>AWS 2</t>
+          <t>AWS 1</t>
         </is>
       </c>
       <c r="B12" s="24" t="inlineStr">
@@ -2565,11 +2542,11 @@
         </is>
       </c>
       <c r="C12" s="19" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/593</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/592</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
@@ -2578,7 +2555,9 @@
         </is>
       </c>
       <c r="F12" s="24" t="n"/>
-      <c r="G12" s="16" t="n"/>
+      <c r="G12" s="19" t="n">
+        <v>2</v>
+      </c>
       <c r="H12" s="38" t="n"/>
       <c r="I12" s="38" t="n"/>
       <c r="J12" s="38" t="n"/>
@@ -2602,20 +2581,20 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>DSA 3 &amp; 4</t>
+          <t>AWS 2</t>
         </is>
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>DevOps: DSA 3 &amp; 4 (New)</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C13" s="19" t="n">
-        <v>672</v>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/672</t>
+        <v>593</v>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/593</t>
         </is>
       </c>
       <c r="E13" s="24" t="inlineStr">
@@ -2648,25 +2627,25 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>DSA 4</t>
+          <t>DSA 3 &amp; 4</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>DevOps: DSA 4 (Feb24 + Mar24)</t>
+          <t>DevOps: DSA 3 &amp; 4 (New)</t>
         </is>
       </c>
       <c r="C14" s="19" t="n">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/673</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/672</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Live only once</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -2694,25 +2673,25 @@
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 2</t>
+          <t>DSA 4</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>Devops: Data Structure Algorithms 2</t>
+          <t>DevOps: DSA 4 (Feb24 + Mar24)</t>
         </is>
       </c>
       <c r="C15" s="19" t="n">
-        <v>510</v>
+        <v>673</v>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/510</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/673</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>Live only once</t>
         </is>
       </c>
       <c r="F15" s="24" t="n"/>
@@ -2740,23 +2719,27 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1 &amp; 2</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="inlineStr">
-        <is>
-          <t>DevOps Breaks: DSA 1 &amp; 2</t>
+          <t>Data Structure Algorithms 2</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Devops: Data Structure Algorithms 2</t>
         </is>
       </c>
       <c r="C16" s="19" t="n">
-        <v>641</v>
+        <v>510</v>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/641</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="n"/>
+          <t>https://www.scaler.com/scm/classes/edit-library/510</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
       <c r="F16" s="24" t="n"/>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="38" t="n"/>
@@ -2782,27 +2765,23 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>Foundations &amp; Network Security</t>
+          <t>Data Structure Algorithms 1 &amp; 2</t>
         </is>
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>DevOps: Foundations &amp; Network Security (Jan 2026)</t>
+          <t>DevOps Breaks: DSA 1 &amp; 2</t>
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>764</v>
+        <v>641</v>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/764</t>
-        </is>
-      </c>
-      <c r="E17" s="24" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
+          <t>https://www.scaler.com/scm/classes/edit-library/641</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="n"/>
       <c r="F17" s="24" t="n"/>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="38" t="n"/>
@@ -2828,20 +2807,20 @@
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>OS &amp; Infrastructure Security</t>
+          <t>Foundations &amp; Network Security</t>
         </is>
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>DevOps: OS &amp; Infrastructure Security (Jan 2026)</t>
+          <t>DevOps: Foundations &amp; Network Security (Jan 2026)</t>
         </is>
       </c>
       <c r="C18" s="19" t="n">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/765</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/764</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
@@ -2874,20 +2853,20 @@
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>Web, API, Application (VAPT) &amp; Cloud Security</t>
+          <t>OS &amp; Infrastructure Security</t>
         </is>
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>DevOps: Web, API, Application (VAPT) &amp; Cloud Security (Jan 2026)</t>
+          <t>DevOps: OS &amp; Infrastructure Security (Jan 2026)</t>
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/766</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/765</t>
         </is>
       </c>
       <c r="E19" s="24" t="inlineStr">
@@ -2920,20 +2899,20 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">GRC, SOC &amp; Capstone (Blue + Red Team Integration) </t>
+          <t>Web, API, Application (VAPT) &amp; Cloud Security</t>
         </is>
       </c>
       <c r="B20" s="26" t="inlineStr">
         <is>
-          <t>DevOps: GRC, SOC &amp; Capstone (Blue + Red Team Integration) (Jan 2026)</t>
+          <t>DevOps: Web, API, Application (VAPT) &amp; Cloud Security (Jan 2026)</t>
         </is>
       </c>
       <c r="C20" s="19" t="n">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/767</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/766</t>
         </is>
       </c>
       <c r="E20" s="24" t="inlineStr">
@@ -2964,33 +2943,31 @@
       <c r="Z20" s="38" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Beginner Python </t>
-        </is>
-      </c>
-      <c r="B21" s="35" t="inlineStr">
-        <is>
-          <t>Devops: Beginner Python (NA)</t>
-        </is>
-      </c>
-      <c r="C21" s="28" t="n">
-        <v>497</v>
-      </c>
-      <c r="D21" s="29" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/497</t>
-        </is>
-      </c>
-      <c r="E21" s="35" t="inlineStr">
-        <is>
-          <t>Old</t>
-        </is>
-      </c>
-      <c r="F21" s="35" t="n"/>
-      <c r="G21" s="30" t="n">
-        <v>1</v>
-      </c>
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRC, SOC &amp; Capstone (Blue + Red Team Integration) </t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>DevOps: GRC, SOC &amp; Capstone (Blue + Red Team Integration) (Jan 2026)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>767</v>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/767</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="16" t="n"/>
       <c r="H21" s="38" t="n"/>
       <c r="I21" s="38" t="n"/>
       <c r="J21" s="38" t="n"/>
@@ -3014,20 +2991,20 @@
     <row r="22">
       <c r="A22" s="35" t="inlineStr">
         <is>
-          <t>Beginner Python with Breaks</t>
+          <t xml:space="preserve">Beginner Python </t>
         </is>
       </c>
       <c r="B22" s="35" t="inlineStr">
         <is>
-          <t>Beginner Python (DevOps) with Breaks (NA)</t>
+          <t>Devops: Beginner Python (NA)</t>
         </is>
       </c>
       <c r="C22" s="28" t="n">
-        <v>586</v>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/586</t>
+        <v>497</v>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/497</t>
         </is>
       </c>
       <c r="E22" s="35" t="inlineStr">
@@ -3036,7 +3013,9 @@
         </is>
       </c>
       <c r="F22" s="35" t="n"/>
-      <c r="G22" s="9" t="n"/>
+      <c r="G22" s="30" t="n">
+        <v>1</v>
+      </c>
       <c r="H22" s="38" t="n"/>
       <c r="I22" s="38" t="n"/>
       <c r="J22" s="38" t="n"/>
@@ -3060,20 +3039,20 @@
     <row r="23">
       <c r="A23" s="35" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t>Beginner Python with Breaks</t>
         </is>
       </c>
       <c r="B23" s="35" t="inlineStr">
         <is>
-          <t>DevOps: Data Structure Algorithms 1 (NA)</t>
+          <t>Beginner Python (DevOps) with Breaks (NA)</t>
         </is>
       </c>
       <c r="C23" s="28" t="n">
-        <v>506</v>
+        <v>586</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/506</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/586</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -3082,9 +3061,7 @@
         </is>
       </c>
       <c r="F23" s="35" t="n"/>
-      <c r="G23" s="30" t="n">
-        <v>2</v>
-      </c>
+      <c r="G23" s="9" t="n"/>
       <c r="H23" s="38" t="n"/>
       <c r="I23" s="38" t="n"/>
       <c r="J23" s="38" t="n"/>
@@ -3108,20 +3085,20 @@
     <row r="24">
       <c r="A24" s="35" t="inlineStr">
         <is>
-          <t>Data Stucture and Algorithms 1 with breaks</t>
+          <t>Data Structure Algorithms 1</t>
         </is>
       </c>
       <c r="B24" s="35" t="inlineStr">
         <is>
-          <t>DevOps: DSA 1with Breaks (NA)</t>
+          <t>DevOps: Data Structure Algorithms 1 (NA)</t>
         </is>
       </c>
       <c r="C24" s="28" t="n">
-        <v>587</v>
+        <v>506</v>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/587</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/506</t>
         </is>
       </c>
       <c r="E24" s="35" t="inlineStr">
@@ -3130,7 +3107,9 @@
         </is>
       </c>
       <c r="F24" s="35" t="n"/>
-      <c r="G24" s="9" t="n"/>
+      <c r="G24" s="30" t="n">
+        <v>2</v>
+      </c>
       <c r="H24" s="38" t="n"/>
       <c r="I24" s="38" t="n"/>
       <c r="J24" s="38" t="n"/>
@@ -3154,20 +3133,20 @@
     <row r="25">
       <c r="A25" s="35" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 1</t>
-        </is>
-      </c>
-      <c r="B25" s="34" t="inlineStr">
-        <is>
-          <t>Devops: Linux Shell Scripting and Computer Systems - 1 (NA)</t>
+          <t>Data Stucture and Algorithms 1 with breaks</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>DevOps: DSA 1with Breaks (NA)</t>
         </is>
       </c>
       <c r="C25" s="28" t="n">
-        <v>436</v>
-      </c>
-      <c r="D25" s="29" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/436</t>
+        <v>587</v>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/587</t>
         </is>
       </c>
       <c r="E25" s="35" t="inlineStr">
@@ -3176,9 +3155,7 @@
         </is>
       </c>
       <c r="F25" s="35" t="n"/>
-      <c r="G25" s="28" t="n">
-        <v>2.5</v>
-      </c>
+      <c r="G25" s="9" t="n"/>
       <c r="H25" s="38" t="n"/>
       <c r="I25" s="38" t="n"/>
       <c r="J25" s="38" t="n"/>
@@ -3202,20 +3179,20 @@
     <row r="26">
       <c r="A26" s="35" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 2</t>
+          <t>Linux Shell Scripting and Computer Systems 1</t>
         </is>
       </c>
       <c r="B26" s="34" t="inlineStr">
         <is>
-          <t>Devops: Linux Shell Scripting and Computer Systems - 2 (NA)</t>
+          <t>Devops: Linux Shell Scripting and Computer Systems - 1 (NA)</t>
         </is>
       </c>
       <c r="C26" s="28" t="n">
-        <v>460</v>
+        <v>436</v>
       </c>
       <c r="D26" s="29" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/460</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/436</t>
         </is>
       </c>
       <c r="E26" s="35" t="inlineStr">
@@ -3224,7 +3201,9 @@
         </is>
       </c>
       <c r="F26" s="35" t="n"/>
-      <c r="G26" s="9" t="n"/>
+      <c r="G26" s="28" t="n">
+        <v>2.5</v>
+      </c>
       <c r="H26" s="38" t="n"/>
       <c r="I26" s="38" t="n"/>
       <c r="J26" s="38" t="n"/>
@@ -3248,20 +3227,20 @@
     <row r="27">
       <c r="A27" s="35" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 3</t>
+          <t>Linux Shell Scripting and Computer Systems 2</t>
         </is>
       </c>
       <c r="B27" s="34" t="inlineStr">
         <is>
-          <t>Devops:Linux Shell Scripting and Computer Systems- 3 (NA)</t>
+          <t>Devops: Linux Shell Scripting and Computer Systems - 2 (NA)</t>
         </is>
       </c>
       <c r="C27" s="28" t="n">
-        <v>477</v>
+        <v>460</v>
       </c>
       <c r="D27" s="29" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/477</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/460</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -3299,15 +3278,15 @@
       </c>
       <c r="B28" s="34" t="inlineStr">
         <is>
-          <t>DevOps: Linux 3 (NA)</t>
+          <t>Devops:Linux Shell Scripting and Computer Systems- 3 (NA)</t>
         </is>
       </c>
       <c r="C28" s="28" t="n">
-        <v>654</v>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/654</t>
+        <v>477</v>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/477</t>
         </is>
       </c>
       <c r="E28" s="35" t="inlineStr">
@@ -3340,20 +3319,20 @@
     <row r="29">
       <c r="A29" s="35" t="inlineStr">
         <is>
-          <t>DevOps Tools 1</t>
-        </is>
-      </c>
-      <c r="B29" s="35" t="inlineStr">
-        <is>
-          <t>DevOps Tools -1</t>
+          <t>Linux Shell Scripting and Computer Systems 3</t>
+        </is>
+      </c>
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>DevOps: Linux 3 (NA)</t>
         </is>
       </c>
       <c r="C29" s="28" t="n">
-        <v>509</v>
-      </c>
-      <c r="D29" s="29" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/509</t>
+        <v>654</v>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/654</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -3362,9 +3341,7 @@
         </is>
       </c>
       <c r="F29" s="35" t="n"/>
-      <c r="G29" s="30" t="n">
-        <v>3</v>
-      </c>
+      <c r="G29" s="9" t="n"/>
       <c r="H29" s="38" t="n"/>
       <c r="I29" s="38" t="n"/>
       <c r="J29" s="38" t="n"/>
@@ -3388,20 +3365,20 @@
     <row r="30">
       <c r="A30" s="35" t="inlineStr">
         <is>
-          <t>DevOps Tools 2</t>
+          <t>DevOps Tools 1</t>
         </is>
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>DevOps Tools -2</t>
+          <t>DevOps Tools -1</t>
         </is>
       </c>
       <c r="C30" s="28" t="n">
-        <v>548</v>
+        <v>509</v>
       </c>
       <c r="D30" s="29" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/548</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/509</t>
         </is>
       </c>
       <c r="E30" s="35" t="inlineStr">
@@ -3410,7 +3387,9 @@
         </is>
       </c>
       <c r="F30" s="35" t="n"/>
-      <c r="G30" s="9" t="n"/>
+      <c r="G30" s="30" t="n">
+        <v>3</v>
+      </c>
       <c r="H30" s="38" t="n"/>
       <c r="I30" s="38" t="n"/>
       <c r="J30" s="38" t="n"/>
@@ -3434,25 +3413,25 @@
     <row r="31">
       <c r="A31" s="35" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 3</t>
+          <t>DevOps Tools 2</t>
         </is>
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>Academy: DSA (Oct)</t>
+          <t>DevOps Tools -2</t>
         </is>
       </c>
       <c r="C31" s="28" t="n">
-        <v>277</v>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
+        <v>548</v>
+      </c>
+      <c r="D31" s="29" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/548</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Not In Curriculum</t>
+          <t>Old</t>
         </is>
       </c>
       <c r="F31" s="35" t="n"/>
@@ -3480,31 +3459,29 @@
     <row r="32">
       <c r="A32" s="35" t="inlineStr">
         <is>
-          <t>IaC</t>
+          <t>Data Structure Algorithms 3</t>
         </is>
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>DevOps: IaC (Not in Use)</t>
+          <t>Academy: DSA (Oct)</t>
         </is>
       </c>
       <c r="C32" s="28" t="n">
-        <v>643</v>
-      </c>
-      <c r="D32" s="29" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/643</t>
+        <v>277</v>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/277</t>
         </is>
       </c>
       <c r="E32" s="35" t="inlineStr">
         <is>
-          <t>Old</t>
+          <t>Not In Curriculum</t>
         </is>
       </c>
       <c r="F32" s="35" t="n"/>
-      <c r="G32" s="30" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G32" s="9" t="n"/>
       <c r="H32" s="38" t="n"/>
       <c r="I32" s="38" t="n"/>
       <c r="J32" s="38" t="n"/>
@@ -3528,16 +3505,30 @@
     <row r="33">
       <c r="A33" s="35" t="inlineStr">
         <is>
-          <t>System Design</t>
-        </is>
-      </c>
-      <c r="B33" s="35" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="35" t="n"/>
-      <c r="E33" s="35" t="n"/>
+          <t>IaC</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>DevOps: IaC (Not in Use)</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="n">
+        <v>643</v>
+      </c>
+      <c r="D33" s="29" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/643</t>
+        </is>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>Old</t>
+        </is>
+      </c>
       <c r="F33" s="35" t="n"/>
       <c r="G33" s="30" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="H33" s="38" t="n"/>
       <c r="I33" s="38" t="n"/>
@@ -3562,7 +3553,7 @@
     <row r="34">
       <c r="A34" s="35" t="inlineStr">
         <is>
-          <t>Adv DSA</t>
+          <t>System Design</t>
         </is>
       </c>
       <c r="B34" s="35" t="n"/>
@@ -3571,7 +3562,7 @@
       <c r="E34" s="35" t="n"/>
       <c r="F34" s="35" t="n"/>
       <c r="G34" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34" s="38" t="n"/>
       <c r="I34" s="38" t="n"/>
@@ -3596,7 +3587,7 @@
     <row r="35">
       <c r="A35" s="35" t="inlineStr">
         <is>
-          <t>Ml Ops</t>
+          <t>Adv DSA</t>
         </is>
       </c>
       <c r="B35" s="35" t="n"/>
@@ -3605,7 +3596,7 @@
       <c r="E35" s="35" t="n"/>
       <c r="F35" s="35" t="n"/>
       <c r="G35" s="30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H35" s="38" t="n"/>
       <c r="I35" s="38" t="n"/>
@@ -3630,29 +3621,17 @@
     <row r="36">
       <c r="A36" s="35" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 1</t>
-        </is>
-      </c>
-      <c r="B36" s="34" t="inlineStr">
-        <is>
-          <t>DevOps: Linux 1 (New) (NA)</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="n">
-        <v>650</v>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/650</t>
-        </is>
-      </c>
-      <c r="E36" s="35" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
+          <t>Ml Ops</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="35" t="n"/>
       <c r="F36" s="35" t="n"/>
-      <c r="G36" s="9" t="n"/>
+      <c r="G36" s="30" t="n">
+        <v>1</v>
+      </c>
       <c r="H36" s="38" t="n"/>
       <c r="I36" s="38" t="n"/>
       <c r="J36" s="38" t="n"/>
@@ -3676,20 +3655,20 @@
     <row r="37">
       <c r="A37" s="35" t="inlineStr">
         <is>
-          <t>Linux Shell Scripting and Computer Systems 2</t>
+          <t>Linux Shell Scripting and Computer Systems 1</t>
         </is>
       </c>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>DevOps: Linux 2 (New) (NA)</t>
+          <t>DevOps: Linux 1 (New) (NA)</t>
         </is>
       </c>
       <c r="C37" s="28" t="n">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/651</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/650</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
@@ -3720,13 +3699,31 @@
       <c r="Z37" s="38" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="36" t="n"/>
-      <c r="B38" s="36" t="n"/>
-      <c r="C38" s="36" t="n"/>
-      <c r="D38" s="36" t="n"/>
-      <c r="E38" s="36" t="n"/>
-      <c r="F38" s="36" t="n"/>
-      <c r="G38" s="4" t="n"/>
+      <c r="A38" s="35" t="inlineStr">
+        <is>
+          <t>Linux Shell Scripting and Computer Systems 2</t>
+        </is>
+      </c>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>DevOps: Linux 2 (New) (NA)</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n">
+        <v>651</v>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/651</t>
+        </is>
+      </c>
+      <c r="E38" s="35" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F38" s="35" t="n"/>
+      <c r="G38" s="9" t="n"/>
       <c r="H38" s="38" t="n"/>
       <c r="I38" s="38" t="n"/>
       <c r="J38" s="38" t="n"/>
@@ -3748,6 +3745,13 @@
       <c r="Z38" s="38" t="n"/>
     </row>
     <row r="39">
+      <c r="A39" s="36" t="n"/>
+      <c r="B39" s="36" t="n"/>
+      <c r="C39" s="36" t="n"/>
+      <c r="D39" s="36" t="n"/>
+      <c r="E39" s="36" t="n"/>
+      <c r="F39" s="36" t="n"/>
+      <c r="G39" s="4" t="n"/>
       <c r="H39" s="38" t="n"/>
       <c r="I39" s="38" t="n"/>
       <c r="J39" s="38" t="n"/>
@@ -24095,6 +24099,27 @@
       <c r="X1007" s="38" t="n"/>
       <c r="Y1007" s="38" t="n"/>
       <c r="Z1007" s="38" t="n"/>
+    </row>
+    <row r="1008">
+      <c r="H1008" s="38" t="n"/>
+      <c r="I1008" s="38" t="n"/>
+      <c r="J1008" s="38" t="n"/>
+      <c r="K1008" s="38" t="n"/>
+      <c r="L1008" s="38" t="n"/>
+      <c r="M1008" s="38" t="n"/>
+      <c r="N1008" s="38" t="n"/>
+      <c r="O1008" s="38" t="n"/>
+      <c r="P1008" s="38" t="n"/>
+      <c r="Q1008" s="38" t="n"/>
+      <c r="R1008" s="38" t="n"/>
+      <c r="S1008" s="38" t="n"/>
+      <c r="T1008" s="38" t="n"/>
+      <c r="U1008" s="38" t="n"/>
+      <c r="V1008" s="38" t="n"/>
+      <c r="W1008" s="38" t="n"/>
+      <c r="X1008" s="38" t="n"/>
+      <c r="Y1008" s="38" t="n"/>
+      <c r="Z1008" s="38" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Add NV Contests library row for Classical ML 2 (DSML)
Classical ML 1 already resolved to NV Contests (338) as its sole
candidate. Classical ML 2 had no row at all — added one alongside
it, same library, matching the DA ML 1 / DA ML 2 pattern already
present in this sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2096,25 +2096,25 @@
       <c r="Z1" s="38" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Linux Shell Scripting and Computer Systems 2</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -3626,7 +3626,11 @@
       </c>
       <c r="B36" s="35" t="n"/>
       <c r="C36" s="35" t="n"/>
-      <c r="D36" s="35" t="n"/>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/650</t>
+        </is>
+      </c>
       <c r="E36" s="35" t="n"/>
       <c r="F36" s="35" t="n"/>
       <c r="G36" s="30" t="n">
@@ -24167,7 +24171,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z44"/>
+  <dimension ref="A1:Z45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="43" customWidth="1" style="46" min="1" max="1"/>
@@ -25164,20 +25168,20 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="0" t="inlineStr">
-        <is>
-          <t>DA ML 1</t>
-        </is>
-      </c>
-      <c r="B42" s="0" t="inlineStr">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Classical ML 2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C42" s="0" t="n">
+      <c r="C42" t="n">
         <v>338</v>
       </c>
-      <c r="D42" s="0" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
@@ -25186,7 +25190,7 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>DA ML 2</t>
+          <t>DA ML 1</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
@@ -25206,7 +25210,7 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>Advanced SQL</t>
+          <t>DA ML 2</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -25218,6 +25222,26 @@
         <v>338</v>
       </c>
       <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>Advanced SQL</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="n">
+        <v>338</v>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>

</xml_diff>

<commit_message>
Fix CCT dropdown search name for Linux 2 NV Contests entry
The library react-select in schedule_creator.py matches by exact
displayed text, not library ID. Scaler shows this particular contest
inside library 338 as "Linux Certification Contest", not the generic
"NV Contests" label used by other modules sharing that same library —
searching "NV Contests" would have found nothing or picked the wrong
option. ID/link unchanged, only the Library Name (search term) fixed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>NV Contests</t>
+          <t>Linux Certification Contest</t>
         </is>
       </c>
       <c r="C2" s="0" t="n">
@@ -25168,20 +25168,20 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>Classical ML 2</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>NV Contests</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>

</xml_diff>

<commit_message>
Add per-module skill-eval checkbox label override
For DevOps "Linux Shell Scripting and Computer Systems 2", the
Mandatory Skill Evaluation checkbox Scaler shows is literally labeled
"Linux Certification Contest" — no words in common with the module
name, so the existing module-name-based checkbox matching in
_check_skill_eval_checkbox would silently tick the wrong contest
(library 338/NV Contests holds a dozen+ unrelated contest sessions).

Adds an optional "Skill Eval Label" column (SheetSpec.skill_eval_col,
LibraryMatch.skill_eval_label) that overrides the checkbox match
target when set, falling back to the module name exactly as before
everywhere it's unset. Verified AWS 1 and other existing rows are
unaffected (skill_eval_label resolves to None for them).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2075,7 +2075,11 @@
           <t>Months</t>
         </is>
       </c>
-      <c r="H1" s="38" t="n"/>
+      <c r="H1" s="38" t="inlineStr">
+        <is>
+          <t>Skill Eval Label</t>
+        </is>
+      </c>
       <c r="I1" s="38" t="n"/>
       <c r="J1" s="38" t="n"/>
       <c r="K1" s="38" t="n"/>
@@ -2117,6 +2121,11 @@
       <c r="E2" s="0" t="inlineStr">
         <is>
           <t>Live</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Linux Certification Contest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Library Name for Linux 2 back to "NV Contests"
Screenshot from the live Schedule Classes page showed the library
react-select returning "No matching libraries found" for "Linux
Certification Contest" — that's the skill-eval checkbox label, not
the library dropdown's option text. The dropdown itself must search
"NV Contests" (same as every other module sharing library 338); the
skill_eval_label override added in ab8cf74 already correctly targets
"Linux Certification Contest" for the checkbox step.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2107,7 +2107,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>Linux Certification Contest</t>
+          <t>NV Contests</t>
         </is>
       </c>
       <c r="C2" s="0" t="n">
@@ -2123,7 +2123,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>Linux Certification Contest</t>
         </is>

</xml_diff>

<commit_message>
Add skill-eval checkbox override for Academy Back-end development
Module already existed (row 76) resolving to NV Contests (338) with
no ambiguity — no new row needed. Adds the same skill_eval_col
mechanism used for DevOps Linux 2 (see commit ab8cf74): Scaler's
Mandatory Skill Evaluation checkbox for this module is labeled
"Back-end development- Neovarsity contest", not the generic module
name, so without the override the auto-matching would tick the wrong
contest among the many sharing library 338.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -602,6 +602,11 @@
           <t>Num Attempts</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Skill Eval Label</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1969,6 +1974,11 @@
       <c r="C76" s="0" t="inlineStr">
         <is>
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Back-end development- Neovarsity contest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch DSML Computer Vision to shared NV Contests library 338
Was previously mapped to a dedicated library (ID 60), which had
worked in a run earlier today. Switched to the shared NV Contests
library (338) since the specific contest "DSML Module Test: Computer
Vision (No Class Today)" lives there, not in library 60 — confirmed
with the operator before changing since library 60 was tested-working.
Added the skill_eval_col override to the DSML sheet (same mechanism
as DevOps/Academy) so the checkbox step targets that exact contest
name instead of relying on module-name substring matching.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -602,7 +602,7 @@
           <t>Num Attempts</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Skill Eval Label</t>
         </is>
@@ -1976,7 +1976,7 @@
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>Back-end development- Neovarsity contest</t>
         </is>
@@ -24234,7 +24234,11 @@
           <t>Months</t>
         </is>
       </c>
-      <c r="H1" s="37" t="n"/>
+      <c r="H1" s="37" t="inlineStr">
+        <is>
+          <t>Skill Eval Label</t>
+        </is>
+      </c>
       <c r="I1" s="37" t="n"/>
       <c r="J1" s="37" t="n"/>
       <c r="K1" s="37" t="n"/>
@@ -24870,11 +24874,16 @@
         </is>
       </c>
       <c r="C30" s="40" t="n">
-        <v>60</v>
+        <v>338</v>
       </c>
       <c r="D30" s="41" t="inlineStr">
         <is>
-          <t>https://www.scaler.com/scm/classes/edit-library/60</t>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>DSML Module Test: Computer Vision (No Class Today)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Disambiguate DevOps DSA 1/2/3 from Academy's same-named modules
Data Structure Algorithms 1/2/3 existed as module names in both the
Academy and DevOps sheets. While resolve() itself is program-scoped
and unambiguous, identical module names across programs risk
colliding in the Google Sheets tracker upsert (_find_module_row
matches on Module Name column A only, not program) and are confusing
in the operator-facing module picker. Suffixed the DevOps rows with
"(DevOps)" — same disambiguation pattern already used for AIML
modules like "Basics of GenAI and AI Agents (AIML)"; the suffix is
stripped automatically before skill-eval checkbox matching.

Academy's DSA 1/2/3/4 rows are untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -2234,7 +2234,7 @@
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t>Data Structure Algorithms 1 (DevOps)</t>
         </is>
       </c>
       <c r="B5" s="24" t="inlineStr">
@@ -2280,7 +2280,7 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t>Data Structure Algorithms 1 (DevOps)</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
@@ -2738,7 +2738,7 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 2</t>
+          <t>Data Structure Algorithms 2 (DevOps)</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
@@ -3104,7 +3104,7 @@
     <row r="24">
       <c r="A24" s="35" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 1</t>
+          <t>Data Structure Algorithms 1 (DevOps)</t>
         </is>
       </c>
       <c r="B24" s="35" t="inlineStr">
@@ -3478,7 +3478,7 @@
     <row r="32">
       <c r="A32" s="35" t="inlineStr">
         <is>
-          <t>Data Structure Algorithms 3</t>
+          <t>Data Structure Algorithms 3 (DevOps)</t>
         </is>
       </c>
       <c r="B32" s="35" t="inlineStr">
@@ -24881,7 +24881,7 @@
           <t>https://www.scaler.com/scm/classes/edit-library/338</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="0" t="inlineStr">
         <is>
           <t>DSML Module Test: Computer Vision (No Class Today)</t>
         </is>

</xml_diff>

<commit_message>
Add Academy module: AI & Agents: From Talking to AI to Building One
New module, maps to NV Contests (338), with skill-eval checkbox
override set to the exact contest name in Scaler ("...Contest" suffix)
per the standard pattern for shared-library modules.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Library__All_Programs.xlsx
+++ b/data/Library__All_Programs.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z76"/>
+  <dimension ref="A1:Z77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="40.88" customWidth="1" style="46" min="1" max="1"/>
@@ -1979,6 +1979,28 @@
       <c r="E76" s="0" t="inlineStr">
         <is>
           <t>Back-end development- Neovarsity contest</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>AI &amp; Agents: From Talking to AI to Building One</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>NV Contests</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/scm/classes/edit-library/338</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>AI &amp; Agents: From Talking to AI to Building One Contest</t>
         </is>
       </c>
     </row>

</xml_diff>